<commit_message>
excel name on exporting is set
</commit_message>
<xml_diff>
--- a/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_BatchSA1_Attendance.xlsx
+++ b/backend/exports/attendance/ComputerEngineering_2026-2027_A_COA_BatchSA1_Attendance.xlsx
@@ -610,7 +610,7 @@
         <v>12</v>
       </c>
       <c r="D7" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
@@ -658,7 +658,7 @@
         <v>12</v>
       </c>
       <c r="D10" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -927,6 +927,6 @@
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>